<commit_message>
corregida frecuencia de muestreo
</commit_message>
<xml_diff>
--- a/Otros/Pruebas/Python/Finales/data/RESULTADOS.xlsx
+++ b/Otros/Pruebas/Python/Finales/data/RESULTADOS.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BloodPressure_v1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BloodPressure_v2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BloodPressure_v1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BloodPressure_v2" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
@@ -99,6 +99,74 @@
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -369,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.88671875" customWidth="1" style="6" min="1" max="9"/>
@@ -1034,17 +1102,14 @@
       <c r="C20" t="n">
         <v>18</v>
       </c>
-      <c r="D20">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E20">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="F20">
-        <f>NA()</f>
-        <v/>
+      <c r="D20" t="n">
+        <v>133</v>
+      </c>
+      <c r="E20" t="n">
+        <v>107</v>
+      </c>
+      <c r="F20" t="n">
+        <v>85</v>
       </c>
       <c r="G20" t="n">
         <v>135</v>
@@ -1062,11 +1127,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Maez</t>
+          <t>Andres</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D21">
         <f>NA()</f>
@@ -1081,13 +1146,13 @@
         <v/>
       </c>
       <c r="G21" t="n">
-        <v>116</v>
+        <v>144</v>
       </c>
       <c r="H21" t="n">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="I21" t="n">
-        <v>54</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22">
@@ -1096,36 +1161,331 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>Andres</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>20</v>
+      </c>
+      <c r="D22" t="n">
+        <v>122</v>
+      </c>
+      <c r="E22" t="n">
+        <v>114</v>
+      </c>
+      <c r="F22" t="n">
+        <v>75</v>
+      </c>
+      <c r="G22" t="n">
+        <v>131</v>
+      </c>
+      <c r="H22" t="n">
+        <v>77</v>
+      </c>
+      <c r="I22" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Andres</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>21</v>
+      </c>
+      <c r="D23">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="E23">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="F23">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="G23" t="n">
+        <v>130</v>
+      </c>
+      <c r="H23" t="n">
+        <v>85</v>
+      </c>
+      <c r="I23" t="n">
+        <v>67</v>
+      </c>
+      <c r="O23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Andres</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>22</v>
+      </c>
+      <c r="D24">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="E24">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="F24">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="G24" t="n">
+        <v>131</v>
+      </c>
+      <c r="H24" t="n">
+        <v>86</v>
+      </c>
+      <c r="I24" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Andres</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>23</v>
+      </c>
+      <c r="D25">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="E25">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="F25">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="G25" t="n">
+        <v>127</v>
+      </c>
+      <c r="H25" t="n">
+        <v>82</v>
+      </c>
+      <c r="I25" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Andres</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>24</v>
+      </c>
+      <c r="D26">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="E26">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="F26">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="G26" t="n">
+        <v>132</v>
+      </c>
+      <c r="H26" t="n">
+        <v>80</v>
+      </c>
+      <c r="I26" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Andres</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>25</v>
+      </c>
+      <c r="D27">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="E27">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="F27">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="G27" t="n">
+        <v>129</v>
+      </c>
+      <c r="H27" t="n">
+        <v>80</v>
+      </c>
+      <c r="I27" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Maez</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="E28">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="F28">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="G28" t="n">
+        <v>116</v>
+      </c>
+      <c r="H28" t="n">
+        <v>65</v>
+      </c>
+      <c r="I28" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Maez</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" t="n">
+        <v>120</v>
+      </c>
+      <c r="E29" t="n">
+        <v>90</v>
+      </c>
+      <c r="F29" t="n">
+        <v>52</v>
+      </c>
+      <c r="G29" t="n">
+        <v>124</v>
+      </c>
+      <c r="H29" t="n">
+        <v>62</v>
+      </c>
+      <c r="I29" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>Pruebas</t>
         </is>
       </c>
-      <c r="C22" t="n">
+      <c r="C30" t="n">
         <v>1</v>
       </c>
-      <c r="D22">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E22">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="F22">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="G22" t="n">
+      <c r="D30">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="E30">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="F30">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="G30" t="n">
         <v>128</v>
       </c>
-      <c r="H22" t="n">
+      <c r="H30" t="n">
         <v>81</v>
       </c>
-      <c r="I22" t="n">
+      <c r="I30" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="23">
-      <c r="O23" s="7" t="n"/>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Pruebas</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" t="n">
+        <v>98</v>
+      </c>
+      <c r="E31" t="n">
+        <v>62</v>
+      </c>
+      <c r="F31" t="n">
+        <v>73</v>
+      </c>
+      <c r="G31" t="n">
+        <v>126</v>
+      </c>
+      <c r="H31" t="n">
+        <v>85</v>
+      </c>
+      <c r="I31" t="n">
+        <v>71</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
ajuste ratios dia sys
</commit_message>
<xml_diff>
--- a/Otros/Pruebas/Python/Finales/data/RESULTADOS.xlsx
+++ b/Otros/Pruebas/Python/Finales/data/RESULTADOS.xlsx
@@ -1148,7 +1148,7 @@
         <v>114</v>
       </c>
       <c r="E4" s="34" t="n">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="F4" s="34" t="n">
         <v>89</v>
@@ -1554,7 +1554,7 @@
         <v>130</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="F11" s="34" t="n">
         <v>77</v>
@@ -1725,10 +1725,10 @@
         <v>12</v>
       </c>
       <c r="D14" s="34" t="n">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="E14" s="34" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F14" s="34" t="n">
         <v>68</v>
@@ -1835,10 +1835,10 @@
         <v>14</v>
       </c>
       <c r="D16" s="34" t="n">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="E16" s="34" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="F16" s="34" t="n">
         <v>65</v>
@@ -1890,10 +1890,10 @@
         <v>15</v>
       </c>
       <c r="D17" s="34" t="n">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="E17" s="34" t="n">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="F17" s="34" t="n">
         <v>70</v>
@@ -1945,10 +1945,10 @@
         <v>16</v>
       </c>
       <c r="D18" s="34" t="n">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="E18" s="34" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="F18" s="34" t="n">
         <v>67</v>
@@ -2003,7 +2003,7 @@
         <v>131</v>
       </c>
       <c r="E19" s="34" t="n">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F19" s="34" t="n">
         <v>65</v>
@@ -2220,7 +2220,7 @@
         <v>21</v>
       </c>
       <c r="D23" s="34" t="n">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="E23" s="34" t="n">
         <v>86</v>
@@ -2276,7 +2276,7 @@
         <v>22</v>
       </c>
       <c r="D24" s="34" t="n">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="E24" s="34" t="n">
         <v>84</v>
@@ -2334,7 +2334,7 @@
         <v>152</v>
       </c>
       <c r="E25" s="34" t="n">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="F25" s="34" t="n">
         <v>89</v>
@@ -2389,7 +2389,7 @@
         <v>124</v>
       </c>
       <c r="E26" s="34" t="n">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="F26" s="34" t="n">
         <v>77</v>
@@ -2444,7 +2444,7 @@
         <v>133</v>
       </c>
       <c r="E27" s="34" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="F27" s="34" t="n">
         <v>79</v>

</xml_diff>

<commit_message>
intento de alguna mejora de bp pero no estoy seguro
</commit_message>
<xml_diff>
--- a/Otros/Pruebas/Python/Finales/data/RESULTADOS.xlsx
+++ b/Otros/Pruebas/Python/Finales/data/RESULTADOS.xlsx
@@ -1061,14 +1061,17 @@
       <c r="C3" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="34" t="n">
-        <v>104</v>
-      </c>
-      <c r="E3" s="34" t="n">
-        <v>86</v>
-      </c>
-      <c r="F3" s="34" t="n">
-        <v>102</v>
+      <c r="D3" s="34">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="E3" s="34">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="F3" s="34">
+        <f>NA()</f>
+        <v/>
       </c>
       <c r="G3" s="34">
         <f>NA()</f>
@@ -1148,7 +1151,7 @@
         <v>114</v>
       </c>
       <c r="E4" s="34" t="n">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="F4" s="34" t="n">
         <v>89</v>
@@ -1202,14 +1205,17 @@
       <c r="C5" s="34" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="34" t="n">
-        <v>123</v>
-      </c>
-      <c r="E5" s="34" t="n">
-        <v>107</v>
-      </c>
-      <c r="F5" s="34" t="n">
-        <v>98</v>
+      <c r="D5" s="34">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="E5" s="34">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="F5" s="34">
+        <f>NA()</f>
+        <v/>
       </c>
       <c r="G5" s="34">
         <f>NA()</f>
@@ -1318,14 +1324,17 @@
       <c r="C7" s="34" t="n">
         <v>5</v>
       </c>
-      <c r="D7" s="34" t="n">
-        <v>110</v>
-      </c>
-      <c r="E7" s="34" t="n">
-        <v>87</v>
-      </c>
-      <c r="F7" s="34" t="n">
-        <v>71</v>
+      <c r="D7" s="34">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="E7" s="34">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="F7" s="34">
+        <f>NA()</f>
+        <v/>
       </c>
       <c r="G7" s="34">
         <f>NA()</f>
@@ -1376,14 +1385,17 @@
       <c r="C8" s="34" t="n">
         <v>6</v>
       </c>
-      <c r="D8" s="34" t="n">
-        <v>113</v>
-      </c>
-      <c r="E8" s="34" t="n">
-        <v>95</v>
-      </c>
-      <c r="F8" s="34" t="n">
-        <v>77</v>
+      <c r="D8" s="34">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="E8" s="34">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="F8" s="34">
+        <f>NA()</f>
+        <v/>
       </c>
       <c r="G8" s="34">
         <f>NA()</f>
@@ -1434,14 +1446,17 @@
       <c r="C9" s="34" t="n">
         <v>7</v>
       </c>
-      <c r="D9" s="34" t="n">
-        <v>126</v>
-      </c>
-      <c r="E9" s="34" t="n">
-        <v>84</v>
-      </c>
-      <c r="F9" s="34" t="n">
-        <v>77</v>
+      <c r="D9" s="34">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="E9" s="34">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="F9" s="34">
+        <f>NA()</f>
+        <v/>
       </c>
       <c r="G9" s="34">
         <f>NA()</f>
@@ -1608,14 +1623,17 @@
       <c r="C12" s="34" t="n">
         <v>10</v>
       </c>
-      <c r="D12" s="34" t="n">
-        <v>134</v>
-      </c>
-      <c r="E12" s="34" t="n">
-        <v>94</v>
-      </c>
-      <c r="F12" s="34" t="n">
-        <v>76</v>
+      <c r="D12" s="34">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="E12" s="34">
+        <f>NA()</f>
+        <v/>
+      </c>
+      <c r="F12" s="34">
+        <f>NA()</f>
+        <v/>
       </c>
       <c r="G12" s="34">
         <f>NA()</f>
@@ -1666,17 +1684,14 @@
       <c r="C13" s="34" t="n">
         <v>11</v>
       </c>
-      <c r="D13" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E13" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="F13" s="34">
-        <f>NA()</f>
-        <v/>
+      <c r="D13" s="34" t="n">
+        <v>98</v>
+      </c>
+      <c r="E13" s="34" t="n">
+        <v>71</v>
+      </c>
+      <c r="F13" s="34" t="n">
+        <v>79</v>
       </c>
       <c r="G13" s="34" t="n">
         <v>126</v>
@@ -1728,7 +1743,7 @@
         <v>124</v>
       </c>
       <c r="E14" s="34" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F14" s="34" t="n">
         <v>68</v>
@@ -1838,7 +1853,7 @@
         <v>114</v>
       </c>
       <c r="E16" s="34" t="n">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="F16" s="34" t="n">
         <v>65</v>
@@ -1893,7 +1908,7 @@
         <v>129</v>
       </c>
       <c r="E17" s="34" t="n">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="F17" s="34" t="n">
         <v>70</v>
@@ -1948,7 +1963,7 @@
         <v>136</v>
       </c>
       <c r="E18" s="34" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F18" s="34" t="n">
         <v>67</v>
@@ -2003,7 +2018,7 @@
         <v>131</v>
       </c>
       <c r="E19" s="34" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F19" s="34" t="n">
         <v>65</v>
@@ -2334,7 +2349,7 @@
         <v>152</v>
       </c>
       <c r="E25" s="34" t="n">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="F25" s="34" t="n">
         <v>89</v>
@@ -2389,7 +2404,7 @@
         <v>124</v>
       </c>
       <c r="E26" s="34" t="n">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="F26" s="34" t="n">
         <v>77</v>
@@ -2444,7 +2459,7 @@
         <v>133</v>
       </c>
       <c r="E27" s="34" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F27" s="34" t="n">
         <v>79</v>
@@ -2495,17 +2510,14 @@
       <c r="C28" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="D28" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E28" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="F28" s="34">
-        <f>NA()</f>
-        <v/>
+      <c r="D28" s="34" t="n">
+        <v>110</v>
+      </c>
+      <c r="E28" s="34" t="n">
+        <v>59</v>
+      </c>
+      <c r="F28" s="34" t="n">
+        <v>57</v>
       </c>
       <c r="G28" s="34" t="n">
         <v>116</v>
@@ -2597,120 +2609,44 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="n">
-        <v>27</v>
-      </c>
-      <c r="B30" s="34" t="inlineStr">
-        <is>
-          <t>Pruebas</t>
-        </is>
-      </c>
-      <c r="C30" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E30" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="F30" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="G30" s="34" t="n">
-        <v>128</v>
-      </c>
-      <c r="H30" s="34" t="n">
-        <v>81</v>
-      </c>
-      <c r="I30" s="34" t="n">
-        <v>60</v>
-      </c>
+      <c r="A30" s="14" t="n"/>
+      <c r="B30" s="34" t="n"/>
+      <c r="C30" s="34" t="n"/>
+      <c r="D30" s="34" t="n"/>
+      <c r="E30" s="34" t="n"/>
+      <c r="F30" s="34" t="n"/>
+      <c r="G30" s="34" t="n"/>
+      <c r="H30" s="34" t="n"/>
+      <c r="I30" s="34" t="n"/>
       <c r="J30" s="34">
         <f>IF(NOT(ISBLANK($A30)), ABS(G30-D30), "")</f>
         <v/>
       </c>
-      <c r="K30" s="15">
-        <f>J30/G30</f>
-        <v/>
-      </c>
-      <c r="L30" s="34">
-        <f>ABS(H30-E30)</f>
-        <v/>
-      </c>
-      <c r="M30" s="15">
-        <f>L30/H30</f>
-        <v/>
-      </c>
-      <c r="N30" s="34">
-        <f>ABS(I30-F30)</f>
-        <v/>
-      </c>
-      <c r="O30" s="15">
-        <f>N30/I30</f>
-        <v/>
-      </c>
+      <c r="K30" s="15" t="n"/>
+      <c r="L30" s="34" t="n"/>
+      <c r="M30" s="15" t="n"/>
+      <c r="N30" s="34" t="n"/>
+      <c r="O30" s="15" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="14" t="n">
-        <v>28</v>
-      </c>
-      <c r="B31" s="34" t="inlineStr">
-        <is>
-          <t>Pruebas</t>
-        </is>
-      </c>
-      <c r="C31" s="34" t="n">
-        <v>2</v>
-      </c>
-      <c r="D31" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E31" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="F31" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="G31" s="34" t="n">
-        <v>126</v>
-      </c>
-      <c r="H31" s="34" t="n">
-        <v>85</v>
-      </c>
-      <c r="I31" s="34" t="n">
-        <v>71</v>
-      </c>
+      <c r="A31" s="14" t="n"/>
+      <c r="B31" s="34" t="n"/>
+      <c r="C31" s="34" t="n"/>
+      <c r="D31" s="34" t="n"/>
+      <c r="E31" s="34" t="n"/>
+      <c r="F31" s="34" t="n"/>
+      <c r="G31" s="34" t="n"/>
+      <c r="H31" s="34" t="n"/>
+      <c r="I31" s="34" t="n"/>
       <c r="J31" s="34">
         <f>IF(NOT(ISBLANK($A31)), ABS(G31-D31), "")</f>
         <v/>
       </c>
-      <c r="K31" s="15">
-        <f>J31/G31</f>
-        <v/>
-      </c>
-      <c r="L31" s="34">
-        <f>ABS(H31-E31)</f>
-        <v/>
-      </c>
-      <c r="M31" s="15">
-        <f>L31/H31</f>
-        <v/>
-      </c>
-      <c r="N31" s="34">
-        <f>ABS(I31-F31)</f>
-        <v/>
-      </c>
-      <c r="O31" s="15">
-        <f>N31/I31</f>
-        <v/>
-      </c>
+      <c r="K31" s="15" t="n"/>
+      <c r="L31" s="34" t="n"/>
+      <c r="M31" s="15" t="n"/>
+      <c r="N31" s="34" t="n"/>
+      <c r="O31" s="15" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="17" t="n"/>

</xml_diff>

<commit_message>
seleccion de mejores metodos bp
</commit_message>
<xml_diff>
--- a/Otros/Pruebas/Python/Finales/data/RESULTADOS.xlsx
+++ b/Otros/Pruebas/Python/Finales/data/RESULTADOS.xlsx
@@ -1061,17 +1061,14 @@
       <c r="C3" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E3" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="F3" s="34">
-        <f>NA()</f>
-        <v/>
+      <c r="D3" s="34" t="n">
+        <v>104</v>
+      </c>
+      <c r="E3" s="34" t="n">
+        <v>86</v>
+      </c>
+      <c r="F3" s="34" t="n">
+        <v>102</v>
       </c>
       <c r="G3" s="34">
         <f>NA()</f>
@@ -1151,10 +1148,10 @@
         <v>114</v>
       </c>
       <c r="E4" s="34" t="n">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="F4" s="34" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G4" s="34">
         <f>NA()</f>
@@ -1205,17 +1202,14 @@
       <c r="C5" s="34" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E5" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="F5" s="34">
-        <f>NA()</f>
-        <v/>
+      <c r="D5" s="34" t="n">
+        <v>123</v>
+      </c>
+      <c r="E5" s="34" t="n">
+        <v>107</v>
+      </c>
+      <c r="F5" s="34" t="n">
+        <v>96</v>
       </c>
       <c r="G5" s="34">
         <f>NA()</f>
@@ -1273,7 +1267,7 @@
         <v>101</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G6" s="34">
         <f>NA()</f>
@@ -1324,17 +1318,14 @@
       <c r="C7" s="34" t="n">
         <v>5</v>
       </c>
-      <c r="D7" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E7" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="F7" s="34">
-        <f>NA()</f>
-        <v/>
+      <c r="D7" s="34" t="n">
+        <v>110</v>
+      </c>
+      <c r="E7" s="34" t="n">
+        <v>87</v>
+      </c>
+      <c r="F7" s="34" t="n">
+        <v>72</v>
       </c>
       <c r="G7" s="34">
         <f>NA()</f>
@@ -1385,17 +1376,14 @@
       <c r="C8" s="34" t="n">
         <v>6</v>
       </c>
-      <c r="D8" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E8" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="F8" s="34">
-        <f>NA()</f>
-        <v/>
+      <c r="D8" s="34" t="n">
+        <v>133</v>
+      </c>
+      <c r="E8" s="34" t="n">
+        <v>95</v>
+      </c>
+      <c r="F8" s="34" t="n">
+        <v>77</v>
       </c>
       <c r="G8" s="34">
         <f>NA()</f>
@@ -1446,17 +1434,14 @@
       <c r="C9" s="34" t="n">
         <v>7</v>
       </c>
-      <c r="D9" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E9" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="F9" s="34">
-        <f>NA()</f>
-        <v/>
+      <c r="D9" s="34" t="n">
+        <v>126</v>
+      </c>
+      <c r="E9" s="34" t="n">
+        <v>84</v>
+      </c>
+      <c r="F9" s="34" t="n">
+        <v>76</v>
       </c>
       <c r="G9" s="34">
         <f>NA()</f>
@@ -1514,7 +1499,7 @@
         <v>86</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G10" s="34">
         <f>NA()</f>
@@ -1572,7 +1557,7 @@
         <v>80</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G11" s="34">
         <f>NA()</f>
@@ -1623,17 +1608,14 @@
       <c r="C12" s="34" t="n">
         <v>10</v>
       </c>
-      <c r="D12" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="E12" s="34">
-        <f>NA()</f>
-        <v/>
-      </c>
-      <c r="F12" s="34">
-        <f>NA()</f>
-        <v/>
+      <c r="D12" s="34" t="n">
+        <v>134</v>
+      </c>
+      <c r="E12" s="34" t="n">
+        <v>94</v>
+      </c>
+      <c r="F12" s="34" t="n">
+        <v>74</v>
       </c>
       <c r="G12" s="34">
         <f>NA()</f>
@@ -1688,10 +1670,10 @@
         <v>98</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="G13" s="34" t="n">
         <v>126</v>
@@ -1746,7 +1728,7 @@
         <v>73</v>
       </c>
       <c r="F14" s="34" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="G14" s="34" t="n">
         <v>120</v>
@@ -1798,10 +1780,10 @@
         <v>130</v>
       </c>
       <c r="E15" s="34" t="n">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="F15" s="34" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G15" s="34" t="n">
         <v>135</v>
@@ -1853,10 +1835,10 @@
         <v>114</v>
       </c>
       <c r="E16" s="34" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="F16" s="34" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G16" s="34" t="n">
         <v>117</v>
@@ -1908,10 +1890,10 @@
         <v>129</v>
       </c>
       <c r="E17" s="34" t="n">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="F17" s="34" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G17" s="34" t="n">
         <v>123</v>
@@ -1963,10 +1945,10 @@
         <v>136</v>
       </c>
       <c r="E18" s="34" t="n">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="F18" s="34" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G18" s="34" t="n">
         <v>134</v>
@@ -2021,7 +2003,7 @@
         <v>81</v>
       </c>
       <c r="F19" s="34" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G19" s="34" t="n">
         <v>136</v>
@@ -2076,7 +2058,7 @@
         <v>82</v>
       </c>
       <c r="F20" s="34" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G20" s="34" t="n">
         <v>135</v>
@@ -2186,7 +2168,7 @@
         <v>91</v>
       </c>
       <c r="F22" s="34" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G22" s="34" t="n">
         <v>131</v>
@@ -2241,7 +2223,7 @@
         <v>86</v>
       </c>
       <c r="F23" s="34" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G23" s="34" t="n">
         <v>130</v>
@@ -2297,7 +2279,7 @@
         <v>84</v>
       </c>
       <c r="F24" s="34" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G24" s="34" t="n">
         <v>131</v>
@@ -2349,7 +2331,7 @@
         <v>152</v>
       </c>
       <c r="E25" s="34" t="n">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="F25" s="34" t="n">
         <v>89</v>
@@ -2404,7 +2386,7 @@
         <v>124</v>
       </c>
       <c r="E26" s="34" t="n">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="F26" s="34" t="n">
         <v>77</v>
@@ -2459,10 +2441,10 @@
         <v>133</v>
       </c>
       <c r="E27" s="34" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="F27" s="34" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G27" s="34" t="n">
         <v>129</v>
@@ -2514,7 +2496,7 @@
         <v>110</v>
       </c>
       <c r="E28" s="34" t="n">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="F28" s="34" t="n">
         <v>57</v>
@@ -2569,10 +2551,10 @@
         <v>134</v>
       </c>
       <c r="E29" s="34" t="n">
-        <v>77</v>
+        <v>45</v>
       </c>
       <c r="F29" s="34" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G29" s="34" t="n">
         <v>124</v>

</xml_diff>